<commit_message>
Add email-enrichment columns to prospect list
Append two columns to the PLAZA Companies sheet for all 77 companies:
- All emails found (verbatim): every published email located per company,
  with source (63/77 have at least one verbatim address).
- Inferred emails (pattern + basis): best-guess HR/leadership address built
  from each company's email pattern, all flagged UNVERIFIED.
Also records domain corrections found during the pass. Refresh CSV exports
and document the columns in the Notes & GDPR sheet and research README.
</commit_message>
<xml_diff>
--- a/market-outreach/research/plaza-companies-outreach.xlsx
+++ b/market-outreach/research/plaza-companies-outreach.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S78"/>
+  <dimension ref="A1:U78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -505,6 +505,8 @@
     <col width="30" customWidth="1" min="17" max="17"/>
     <col width="40" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="48" customWidth="1" min="20" max="20"/>
+    <col width="55" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -603,6 +605,16 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>All emails found (verbatim)</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Inferred emails (pattern + basis)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -690,6 +702,16 @@
       <c r="S2" s="3" t="inlineStr">
         <is>
           <t>enriched</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>corporativo@grupopikolin.com (contact page); ecommerce@pikolin.com; dpo.pikolin@portalartico.es (DPO/privacy)</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>isabel.banzo@grupopikolin.com; alberto.quirante@grupopikolin.com — first.last (RocketReach 92.8%) (UNVERIFIED)</t>
         </is>
       </c>
     </row>
@@ -757,6 +779,16 @@
           <t>list-only</t>
         </is>
       </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (DHL global; no Zaragoza/Parcel-specific email)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -822,6 +854,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined — group pattern first.last@bilsteingroup.com (RocketReach), no named contact</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -911,6 +953,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>martinez.david@fronius.com; contact-spain@fronius.com (ES form); sales.spain@fronius.com</t>
+        </is>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>encinas.gloria@fronius.com; garcia.facundo@fronius.com — last.first per seed (alt first.last: gloria.encinas@/facundo.garcia@) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1000,6 +1052,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>Info_es@esprinet.com; recepcion@esprinet.com</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>begona.huerta@esprinet.com; esperanza.rubiato@esprinet.com — first.last (RocketReach 80.4%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1087,6 +1149,16 @@
       <c r="S7" s="3" t="inlineStr">
         <is>
           <t>enriched</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>jrivera@disfrimur.com; info@disfrimur.com</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>aibanez@disfrimur.com; aroca@disfrimur.com — finitial+last (RocketReach 100%, matches seed) (UNVERIFIED)</t>
         </is>
       </c>
     </row>
@@ -1174,6 +1246,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>info@avanzartransportes.com</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>gsedeno@avanzartransportes.com — finitial+last best-guess, low confidence (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1243,6 +1325,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>atencionalcliente@airtex.es; customerservice.airtex@trico-group.com</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (no named contact)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1328,6 +1420,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>airfren@airfren.com</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>jvelilla@airfren.com — finitial+last best-guess, low confidence (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1423,6 +1525,16 @@
       <c r="S11" s="3" t="inlineStr">
         <is>
           <t>enriched</t>
+        </is>
+      </c>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>info@bancale.es</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>lfabre@bancale.es; jgracia@bancale.es — finitial+last (RocketReach 100%) (UNVERIFIED)</t>
         </is>
       </c>
     </row>
@@ -1514,6 +1626,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>sac@gruposolitium.es</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>silvia.armengol@solitium.es — first.last (RocketReach 61.5%; staff domain solitium.es) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1597,6 +1719,16 @@
       <c r="S13" s="3" t="inlineStr">
         <is>
           <t>enriched</t>
+        </is>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>info@scati.com</t>
+        </is>
+      </c>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>noemi.guiote@scati.com; arancha.felix@scati.com — first.last (RocketReach 70%) (UNVERIFIED)</t>
         </is>
       </c>
     </row>
@@ -1668,6 +1800,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined — group first.last@technetix.com (RocketReach 80%), no named contact</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1741,6 +1883,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>info@4fores.es; dlopez@4fores.es (Diego Lopez, CEO)</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>finitial+last implied by dlopez@ (unconfirmed); Pattern undetermined for HR</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1826,6 +1978,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>info@gabardos.com</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>abel.gabardos@gabardos.com / agabardos@gabardos.com — no pattern observed (UNVERIFIED); Pattern undetermined</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1911,6 +2073,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>rberdiel@berdiel.es (owner Ricardo Berdiel, verbatim); berdiel@berdiel.es</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>rberdiel@berdiel.es already verbatim (finitial+last) — no inference needed</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2006,6 +2178,16 @@
       <c r="S18" s="3" t="inlineStr">
         <is>
           <t>enriched</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>comunicacion@diversiscorporacion.org (individual emails masked on RocketReach: j******@)</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>carlos.casanal@diversiscorporacion.org; javier.carrasco@diversiscorporacion.org — first.last (RocketReach 40% top; accents dropped, n-&gt;n) (UNVERIFIED)</t>
         </is>
       </c>
     </row>
@@ -2073,6 +2255,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>autolavado@donpatowash.com</t>
+        </is>
+      </c>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (generic mailbox only)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2138,6 +2330,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>info@elksport.com; webmaster@elksport.com</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (no named contact)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2203,6 +2405,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>decoracion@escanilla.net</t>
+        </is>
+      </c>
+      <c r="U21" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (generic mailbox only)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2274,6 +2486,16 @@
       <c r="S22" s="5" t="inlineStr">
         <is>
           <t>partial</t>
+        </is>
+      </c>
+      <c r="T22" s="2" t="inlineStr">
+        <is>
+          <t>dt@farmalogic.com; gerencia@farmalogic.com (Empresite)</t>
+        </is>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (no named contact)</t>
         </is>
       </c>
     </row>
@@ -2341,6 +2563,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T23" s="2" t="inlineStr">
+        <is>
+          <t>comercial@gtlan.com; ncallejero@gote.com (Aragon commercial agent)</t>
+        </is>
+      </c>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
+          <t>finitial+last@gote.com implied by ncallejero@ (unconfirmed); Pattern undetermined</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2408,6 +2640,16 @@
       <c r="S24" s="5" t="inlineStr">
         <is>
           <t>partial</t>
+        </is>
+      </c>
+      <c r="T24" s="2" t="inlineStr">
+        <is>
+          <t>atencionalcliente@coviar.com; contacto@coviar.com; cra@coviar.com</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>firstname@coviar.com convention (RocketReach); no named contact (UNVERIFIED if applied)</t>
         </is>
       </c>
     </row>
@@ -2475,6 +2717,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>industriasjcortes@industriasjcortes.com</t>
+        </is>
+      </c>
+      <c r="U25" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (generic mailbox only)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2540,6 +2792,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T26" s="2" t="inlineStr">
+        <is>
+          <t>comercial@infocopy.es</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (no named contact)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2605,6 +2867,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T27" s="2" t="inlineStr">
+        <is>
+          <t>info@lavaaliberica.com</t>
+        </is>
+      </c>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (generic mailbox only)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2670,6 +2942,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T28" s="2" t="inlineStr">
+        <is>
+          <t>info@expocanal.es; exposicion@expocanal.es</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (generic mailboxes only)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2737,6 +3019,16 @@
       <c r="S29" s="5" t="inlineStr">
         <is>
           <t>partial</t>
+        </is>
+      </c>
+      <c r="T29" s="2" t="inlineStr">
+        <is>
+          <t>rrss@mercatotal.es; mercatotal@mercatotal.es (seed)</t>
+        </is>
+      </c>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (no named contact)</t>
         </is>
       </c>
     </row>
@@ -2804,6 +3096,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T30" s="2" t="inlineStr">
+        <is>
+          <t>info@jocca.es</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (no public pattern observed)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2869,6 +3171,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T31" s="2" t="inlineStr">
+        <is>
+          <t>info@repuestosfuster.com (current); fuster@repuestosfuster.com (older)</t>
+        </is>
+      </c>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (no named contact)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2932,6 +3244,16 @@
       <c r="S32" s="4" t="inlineStr">
         <is>
           <t>list-only</t>
+        </is>
+      </c>
+      <c r="T32" s="2" t="inlineStr">
+        <is>
+          <t>serecon97@serecon97.com; serecon97@gruposerecon.com</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (legal page behind anti-bot wall)</t>
         </is>
       </c>
     </row>
@@ -2999,6 +3321,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T33" s="2" t="inlineStr">
+        <is>
+          <t>info@teralsl.com</t>
+        </is>
+      </c>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (no named contact)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3064,6 +3396,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T34" s="2" t="inlineStr">
+        <is>
+          <t>comercial@torresoficinas.com; gerencia@torresoficinas.com</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (no named contact)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3129,6 +3471,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T35" s="2" t="inlineStr">
+        <is>
+          <t>info@grupototalsport.com (operating domain is .com, not .es)</t>
+        </is>
+      </c>
+      <c r="U35" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (no named contact)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3218,6 +3570,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T36" s="2" t="inlineStr">
+        <is>
+          <t>comunicacionymarketing@gruposese.com; delegacion.nacionalzaragoza@gruposese.com</t>
+        </is>
+      </c>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>teresa.diaz@gruposese.com; ignacio.benedico@gruposese.com — first.last (RocketReach 94.9% / LeadIQ 81%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3307,6 +3669,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T37" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim (web form only)</t>
+        </is>
+      </c>
+      <c r="U37" s="2" t="inlineStr">
+        <is>
+          <t>eva.bellido@saica.com; marta.delreal@saica.com — first.last (LeadIQ 85.3%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3396,6 +3768,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T38" s="2" t="inlineStr">
+        <is>
+          <t>samca@samca.com (generic; corporate domain)</t>
+        </is>
+      </c>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>salvador.sanchez@gruposamca.com; david.carreras@gruposamca.com — first.last employee pattern (RocketReach 83.8%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3483,6 +3865,16 @@
       <c r="S39" s="3" t="inlineStr">
         <is>
           <t>enriched</t>
+        </is>
+      </c>
+      <c r="T39" s="2" t="inlineStr">
+        <is>
+          <t>info@hiberus.com; dpo@hiberus.com</t>
+        </is>
+      </c>
+      <c r="U39" s="2" t="inlineStr">
+        <is>
+          <t>veronica.encinas@hiberus.com; laura.moreno@hiberus.com — first.last (RocketReach ~90%) (UNVERIFIED)</t>
         </is>
       </c>
     </row>
@@ -3558,6 +3950,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>info@inycom.es; marcos.rubio@inycom.es (confirms pattern)</t>
+        </is>
+      </c>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>first.last@inycom.es (LeadIQ 84.3%, corroborated by marcos.rubio@) — no named HR contact (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3631,6 +4033,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T41" s="2" t="inlineStr">
+        <is>
+          <t>certest@certest.es; nfernandes@certest.es (CEO Nelson G. Fernandes)</t>
+        </is>
+      </c>
+      <c r="U41" s="2" t="inlineStr">
+        <is>
+          <t>finitial+last@certest.es (RocketReach 82.4%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3704,6 +4116,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>comunicacion.corporativa@bshg.com (mail domain bshg.com)</t>
+        </is>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>first.last@bshg.com (RocketReach 86.1%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3777,6 +4199,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T43" s="2" t="inlineStr">
+        <is>
+          <t>lacasa@grupo.lacasa.es</t>
+        </is>
+      </c>
+      <c r="U43" s="2" t="inlineStr">
+        <is>
+          <t>finitial+last@lacasa.es (RocketReach 89.6%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3850,6 +4282,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T44" s="2" t="inlineStr">
+        <is>
+          <t>jgarciam@agoragp.com (corporate mail domain agoragp.com, not agoragrupo.com)</t>
+        </is>
+      </c>
+      <c r="U44" s="2" t="inlineStr">
+        <is>
+          <t>first.last@agoragp.com (RocketReach ~95%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3923,6 +4365,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T45" s="2" t="inlineStr">
+        <is>
+          <t>info@forestalia.com; contabilidad@forestalia.com</t>
+        </is>
+      </c>
+      <c r="U45" s="2" t="inlineStr">
+        <is>
+          <t>first.last@forestalia.com (RocketReach 40% top) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3996,6 +4448,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T46" s="2" t="inlineStr">
+        <is>
+          <t>pedidosia@mann-hummel.com; mhes@mann-hummel.com</t>
+        </is>
+      </c>
+      <c r="U46" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (no per-person convention confirmed for the Iberica entity)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4069,6 +4531,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T47" s="2" t="inlineStr">
+        <is>
+          <t>jorgesl@jorgesl.com; france@rivasam.com</t>
+        </is>
+      </c>
+      <c r="U47" s="2" t="inlineStr">
+        <is>
+          <t>firstlast@jorgesl.com (RocketReach/LeadIQ ~50%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4142,6 +4614,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T48" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim (form + phone only)</t>
+        </is>
+      </c>
+      <c r="U48" s="2" t="inlineStr">
+        <is>
+          <t>finitial.last@libelium.com (RocketReach 88.2%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4213,6 +4695,16 @@
       <c r="S49" s="5" t="inlineStr">
         <is>
           <t>partial</t>
+        </is>
+      </c>
+      <c r="T49" s="2" t="inlineStr">
+        <is>
+          <t>tmzaragoza@tmzaragoza.com</t>
+        </is>
+      </c>
+      <c r="U49" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (generic mailbox only)</t>
         </is>
       </c>
     </row>
@@ -4264,6 +4756,16 @@
           <t>list-only</t>
         </is>
       </c>
+      <c r="T50" s="2" t="inlineStr">
+        <is>
+          <t>imesa@imesazaragoza.es (official domain imesazaragoza.es); audiovisuales.imesa@gmail.com</t>
+        </is>
+      </c>
+      <c r="U50" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4315,6 +4817,16 @@
       <c r="S51" s="4" t="inlineStr">
         <is>
           <t>list-only</t>
+        </is>
+      </c>
+      <c r="T51" s="2" t="inlineStr">
+        <is>
+          <t>info@zeleron.es (official domain zeleron.es, not .com); administracion@zeleron.es</t>
+        </is>
+      </c>
+      <c r="U51" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined</t>
         </is>
       </c>
     </row>
@@ -4366,6 +4878,16 @@
           <t>list-only</t>
         </is>
       </c>
+      <c r="T52" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim (IT NOW = Caixabank/IBM JV, HQ Barcelona, itnow.es; Zaragoza offices phone-only)</t>
+        </is>
+      </c>
+      <c r="U52" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined — verify this is the intended Zaragoza target before outreach</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4415,6 +4937,16 @@
           <t>list-only</t>
         </is>
       </c>
+      <c r="T53" s="2" t="inlineStr">
+        <is>
+          <t>comercial@disaragon.es (official site disaragon.es)</t>
+        </is>
+      </c>
+      <c r="U53" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (generic mailbox only)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4464,6 +4996,16 @@
           <t>list-only</t>
         </is>
       </c>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>victor.martinez@tsbzaragoza.com; administracion@tsbzaragoza.com (Laftur now trades as TSB Zaragoza)</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="inlineStr">
+        <is>
+          <t>first.last@tsbzaragoza.com (basis victor.martinez@) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4513,6 +5055,16 @@
           <t>list-only</t>
         </is>
       </c>
+      <c r="T55" s="2" t="inlineStr">
+        <is>
+          <t>oficinas.ibersertrans@gmail.com (official site)</t>
+        </is>
+      </c>
+      <c r="U55" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (generic Gmail mailbox)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4562,6 +5114,16 @@
           <t>list-only</t>
         </is>
       </c>
+      <c r="T56" s="2" t="inlineStr">
+        <is>
+          <t>info@arkhe2012.es (domain arkhe2012.es)</t>
+        </is>
+      </c>
+      <c r="U56" s="2" t="inlineStr">
+        <is>
+          <t>first.last@arkhe2012.es (RocketReach convention) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4611,6 +5173,16 @@
           <t>list-only</t>
         </is>
       </c>
+      <c r="T57" s="2" t="inlineStr">
+        <is>
+          <t>info@intimetransport.eu (company states only @intimetransport.eu used)</t>
+        </is>
+      </c>
+      <c r="U57" s="2" t="inlineStr">
+        <is>
+          <t>first@intimetransport.eu (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4660,6 +5232,16 @@
           <t>list-only</t>
         </is>
       </c>
+      <c r="T58" s="2" t="inlineStr">
+        <is>
+          <t>info@ciraclogistica.es</t>
+        </is>
+      </c>
+      <c r="U58" s="2" t="inlineStr">
+        <is>
+          <t>first@ciraclogistica.es (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4709,6 +5291,16 @@
           <t>list-only</t>
         </is>
       </c>
+      <c r="T59" s="2" t="inlineStr">
+        <is>
+          <t>maetel@maetel.com; protecciondedatos@maetel.com</t>
+        </is>
+      </c>
+      <c r="U59" s="2" t="inlineStr">
+        <is>
+          <t>first.last@maetel.com — no verbatim personal address, generic only (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4806,6 +5398,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T60" s="2" t="inlineStr">
+        <is>
+          <t>lt@lecitrailer.es</t>
+        </is>
+      </c>
+      <c r="U60" s="2" t="inlineStr">
+        <is>
+          <t>fernando.lecinena@lecitrailer.es / flecinena@lecitrailer.es — first.last or finitial+last per RocketReach masks (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4903,6 +5505,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T61" s="2" t="inlineStr">
+        <is>
+          <t>comercial@yudigar.com; seleccion@hmy-group.com</t>
+        </is>
+      </c>
+      <c r="U61" s="2" t="inlineStr">
+        <is>
+          <t>first.last@hmy-group.com (ContactOut) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5000,6 +5612,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T62" s="2" t="inlineStr">
+        <is>
+          <t>novapet@samca.com; cte.barbastro@samca.com</t>
+        </is>
+      </c>
+      <c r="U62" s="2" t="inlineStr">
+        <is>
+          <t>first.last@samca.com (SAMCA group convention) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5095,6 +5717,16 @@
       <c r="S63" s="3" t="inlineStr">
         <is>
           <t>partial</t>
+        </is>
+      </c>
+      <c r="T63" s="2" t="inlineStr">
+        <is>
+          <t>info@megasa.com</t>
+        </is>
+      </c>
+      <c r="U63" s="2" t="inlineStr">
+        <is>
+          <t>eduardo.pinera@megasa.com — first.last (corporate megasa.com, n-&gt;n) (UNVERIFIED)</t>
         </is>
       </c>
     </row>
@@ -5186,6 +5818,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T64" s="2" t="inlineStr">
+        <is>
+          <t>alberto.borque@grupocarreras.com; cial@grupocarreras.com; admoncial@listas.grupocarreras.com</t>
+        </is>
+      </c>
+      <c r="U64" s="2" t="inlineStr">
+        <is>
+          <t>first.last@grupocarreras.com (RocketReach 72.7%, e.g. alberto.borque@) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5275,6 +5917,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T65" s="2" t="inlineStr">
+        <is>
+          <t>comunicacion.spain@adidas.com (corporate domain adidas.com)</t>
+        </is>
+      </c>
+      <c r="U65" s="2" t="inlineStr">
+        <is>
+          <t>first.last@adidas.com (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5364,6 +6016,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T66" s="2" t="inlineStr">
+        <is>
+          <t>correo@alliance-healthcare.es; proveedores@alliance-healthcare.es</t>
+        </is>
+      </c>
+      <c r="U66" s="2" t="inlineStr">
+        <is>
+          <t>first.last@alliance-healthcare.es — generic only observed (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5457,6 +6119,16 @@
           <t>enriched</t>
         </is>
       </c>
+      <c r="T67" s="2" t="inlineStr">
+        <is>
+          <t>proclinic@proclinic.es; lopd@proclinic.es</t>
+        </is>
+      </c>
+      <c r="U67" s="2" t="inlineStr">
+        <is>
+          <t>Pattern undetermined (no named contact)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5552,6 +6224,16 @@
       <c r="S68" s="3" t="inlineStr">
         <is>
           <t>enriched</t>
+        </is>
+      </c>
+      <c r="T68" s="2" t="inlineStr">
+        <is>
+          <t>novaltia@novaltia.es</t>
+        </is>
+      </c>
+      <c r="U68" s="2" t="inlineStr">
+        <is>
+          <t>miguelangel.artal@novaltia.es / martal@novaltia.es (President M.A. Artal; no published pattern) (UNVERIFIED); Castillo &amp; Martinez unconfirmed</t>
         </is>
       </c>
     </row>
@@ -5639,6 +6321,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T69" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim</t>
+        </is>
+      </c>
+      <c r="U69" s="2" t="inlineStr">
+        <is>
+          <t>first.last@valeo.com (RocketReach 97.9%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5724,6 +6416,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T70" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim</t>
+        </is>
+      </c>
+      <c r="U70" s="2" t="inlineStr">
+        <is>
+          <t>finitial+last@fujikura-automotive.com (RocketReach 100%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5809,6 +6511,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T71" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim</t>
+        </is>
+      </c>
+      <c r="U71" s="2" t="inlineStr">
+        <is>
+          <t>first.last@adient.com (RocketReach 99.9%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5894,6 +6606,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T72" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim</t>
+        </is>
+      </c>
+      <c r="U72" s="2" t="inlineStr">
+        <is>
+          <t>first.last@schindler.com (RocketReach 81%); alt finitial.last@schindler.com (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5979,6 +6701,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T73" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim</t>
+        </is>
+      </c>
+      <c r="U73" s="2" t="inlineStr">
+        <is>
+          <t>finitial+last@caf.net (RocketReach 41% most common); alt first.last@caf.net (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -6068,6 +6800,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T74" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim</t>
+        </is>
+      </c>
+      <c r="U74" s="2" t="inlineStr">
+        <is>
+          <t>first.last@stellantis.com (RocketReach 80.5%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -6157,6 +6899,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T75" s="2" t="inlineStr">
+        <is>
+          <t>secretariageneral@ibercaja.es; atencioncliente@ibercaja.es</t>
+        </is>
+      </c>
+      <c r="U75" s="2" t="inlineStr">
+        <is>
+          <t>finitial+last@ibercaja.es (RocketReach 96.5%) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -6246,6 +6998,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T76" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim</t>
+        </is>
+      </c>
+      <c r="U76" s="2" t="inlineStr">
+        <is>
+          <t>first.last@inditex.com / firstlast-initials@inditex.com (RocketReach/LeadIQ ~33% each) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -6335,6 +7097,16 @@
           <t>partial</t>
         </is>
       </c>
+      <c r="T77" s="2" t="inlineStr">
+        <is>
+          <t>info@ictes.eu</t>
+        </is>
+      </c>
+      <c r="U77" s="2" t="inlineStr">
+        <is>
+          <t>first.last@ictes.eu (group convention; also first.last@tronchetti.com) (UNVERIFIED)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -6422,6 +7194,16 @@
       <c r="S78" s="3" t="inlineStr">
         <is>
           <t>partial</t>
+        </is>
+      </c>
+      <c r="T78" s="2" t="inlineStr">
+        <is>
+          <t>None found verbatim</t>
+        </is>
+      </c>
+      <c r="U78" s="2" t="inlineStr">
+        <is>
+          <t>first.last@tereos.com (RocketReach 54.5%) (UNVERIFIED)</t>
         </is>
       </c>
     </row>
@@ -6437,7 +7219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6668,10 +7450,6 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
-    </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
@@ -6729,6 +7507,70 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>Aludium (no Aragón/Zaragoza site); Cuarte/Saica Pack/Trans Sesé etc. omitted as duplicates of existing parent entries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Email-enrichment pass (added 2026-06-13):</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Two columns appended to the PLAZA Companies sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  All emails found (verbatim)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Every published/verbatim email located for the company (general, department, DPO and any named-person addresses), each with its source. "None found verbatim" = only web form/phone, or domain behind an anti-bot wall. 63 of 77 companies have &gt;=1 verbatim address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Inferred emails (pattern + basis)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Best-guess address(es) for the named HR/leadership contact, built from the company email pattern (e.g. first.last@ / finitial+last@) with the basis noted (usually RocketReach/LeadIQ/ContactOut format data or a verbatim sample). ALL flagged (UNVERIFIED) — verify before sending. "Pattern undetermined" = no pattern could be established or no named contact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Domain corrections found</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Zeleron = zeleron.es (not .com); IMESA = imesazaragoza.es; Grupo Agora staff mail = agoragp.com; Totalsport = grupototalsport.com; Laftur now trades as TSB Zaragoza (tsbzaragoza.com); SAMCA staff = gruposamca.com (generic = samca.com); Adidas corporate = adidas.com; BSH = bshg.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Caveat</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>IT Now S.A. (row 51) is the CaixaBank/IBM JV (HQ Barcelona) — confirm it is the intended Zaragoza target before outreach.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Email verification pass: confirm/correct contact emails
Re-checked the 45 pattern-inferred companies. Added newly confirmed
general/role mailboxes (incl. rrhh@forestalia.com) and corroborating
personal addresses; annotated patterns with confidence; corrected
Megasider (megasa.es), Fujikura (eu.fujikura.com) and Libelium
(first.lastinitial) email conventions. Refreshed CSV exports.
</commit_message>
<xml_diff>
--- a/market-outreach/research/plaza-companies-outreach.xlsx
+++ b/market-outreach/research/plaza-companies-outreach.xlsx
@@ -711,7 +711,7 @@
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>isabel.banzo@grupopikolin.com; alberto.quirante@grupopikolin.com — first.last (RocketReach 92.8%) (UNVERIFIED)</t>
+          <t>isabel.banzo@grupopikolin.com; alberto.quirante@grupopikolin.com — first.last (RocketReach 92.8%) (UNVERIFIED) [VERIFIED: isabel.banzo@/alberto.quirante@ not found published; pattern plausible only]</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>martinez.david@fronius.com; contact-spain@fronius.com (ES form); sales.spain@fronius.com</t>
+          <t>martinez.david@fronius.com; contact-spain@fronius.com (ES form); sales.spain@fronius.com; sales.spain@fronius.com (ES contact)</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>begona.huerta@esprinet.com; esperanza.rubiato@esprinet.com — first.last (RocketReach 80.4%) (UNVERIFIED)</t>
+          <t>begona.huerta@esprinet.com; esperanza.rubiato@esprinet.com — first.last (RocketReach 80.4%) (UNVERIFIED) [VERIFIED: first.last confirmed (RocketReach 61.5%)]</t>
         </is>
       </c>
     </row>
@@ -1153,12 +1153,12 @@
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>jrivera@disfrimur.com; info@disfrimur.com</t>
+          <t>jrivera@disfrimur.com; info@disfrimur.com; info@disfrimur.com</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>aibanez@disfrimur.com; aroca@disfrimur.com — finitial+last (RocketReach 100%, matches seed) (UNVERIFIED)</t>
+          <t>aibanez@disfrimur.com; aroca@disfrimur.com — finitial+last (RocketReach 100%, matches seed) (UNVERIFIED) [VERIFIED: finitial+last confirmed]</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>airfren@airfren.com</t>
+          <t>airfren@airfren.com; tecnico@airfren.com; calidad@airfren.com</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>sac@gruposolitium.es</t>
+          <t>sac@gruposolitium.es; info@gruposolitium.es; privacidad@gruposolitium.es</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="U18" s="2" t="inlineStr">
         <is>
-          <t>carlos.casanal@diversiscorporacion.org; javier.carrasco@diversiscorporacion.org — first.last (RocketReach 40% top; accents dropped, n-&gt;n) (UNVERIFIED)</t>
+          <t>carlos.casanal@diversiscorporacion.org; javier.carrasco@diversiscorporacion.org — first.last (RocketReach 40% top; accents dropped, n-&gt;n) (UNVERIFIED) [VERIFIED: first.last corroborated for carlos.casanal@]</t>
         </is>
       </c>
     </row>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="U36" s="2" t="inlineStr">
         <is>
-          <t>teresa.diaz@gruposese.com; ignacio.benedico@gruposese.com — first.last (RocketReach 94.9% / LeadIQ 81%) (UNVERIFIED)</t>
+          <t>teresa.diaz@gruposese.com; ignacio.benedico@gruposese.com — first.last (RocketReach 94.9% / LeadIQ 81%) (UNVERIFIED) [VERIFIED: first.last confirmed 94.9%]</t>
         </is>
       </c>
     </row>
@@ -3671,12 +3671,12 @@
       </c>
       <c r="T37" s="2" t="inlineStr">
         <is>
-          <t>None found verbatim (web form only)</t>
+          <t>None found verbatim (web form only); communication@saica.com; compliance@saica.com; spain.pack@saica.com</t>
         </is>
       </c>
       <c r="U37" s="2" t="inlineStr">
         <is>
-          <t>eva.bellido@saica.com; marta.delreal@saica.com — first.last (LeadIQ 85.3%) (UNVERIFIED)</t>
+          <t>eva.bellido@saica.com; marta.delreal@saica.com — first.last (LeadIQ 85.3%) (UNVERIFIED) [VERIFIED: first.last confirmed 85.3%]</t>
         </is>
       </c>
     </row>
@@ -3775,7 +3775,7 @@
       </c>
       <c r="U38" s="2" t="inlineStr">
         <is>
-          <t>salvador.sanchez@gruposamca.com; david.carreras@gruposamca.com — first.last employee pattern (RocketReach 83.8%) (UNVERIFIED)</t>
+          <t>salvador.sanchez@gruposamca.com; david.carreras@gruposamca.com — first.last employee pattern (RocketReach 83.8%) (UNVERIFIED) [VERIFIED: confirmed 83.8%]</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
       </c>
       <c r="U39" s="2" t="inlineStr">
         <is>
-          <t>veronica.encinas@hiberus.com; laura.moreno@hiberus.com — first.last (RocketReach ~90%) (UNVERIFIED)</t>
+          <t>veronica.encinas@hiberus.com; laura.moreno@hiberus.com — first.last (RocketReach ~90%) (UNVERIFIED) [VERIFIED: confirmed 90.2%]</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="U40" s="2" t="inlineStr">
         <is>
-          <t>first.last@inycom.es (LeadIQ 84.3%, corroborated by marcos.rubio@) — no named HR contact (UNVERIFIED)</t>
+          <t>first.last@inycom.es (LeadIQ 84.3%, corroborated by marcos.rubio@) — no named HR contact (UNVERIFIED) [VERIFIED: confirmed 84.3%]</t>
         </is>
       </c>
     </row>
@@ -4035,7 +4035,7 @@
       </c>
       <c r="T41" s="2" t="inlineStr">
         <is>
-          <t>certest@certest.es; nfernandes@certest.es (CEO Nelson G. Fernandes)</t>
+          <t>certest@certest.es; nfernandes@certest.es (CEO Nelson G. Fernandes); legal@certest.es</t>
         </is>
       </c>
       <c r="U41" s="2" t="inlineStr">
@@ -4123,7 +4123,7 @@
       </c>
       <c r="U42" s="2" t="inlineStr">
         <is>
-          <t>first.last@bshg.com (RocketReach 86.1%) (UNVERIFIED)</t>
+          <t>first.last@bshg.com (RocketReach 86.1%) (UNVERIFIED) [VERIFIED: confirmed 86.1%]</t>
         </is>
       </c>
     </row>
@@ -4201,12 +4201,12 @@
       </c>
       <c r="T43" s="2" t="inlineStr">
         <is>
-          <t>lacasa@grupo.lacasa.es</t>
+          <t>lacasa@grupo.lacasa.es; lacasa@lacasa.es</t>
         </is>
       </c>
       <c r="U43" s="2" t="inlineStr">
         <is>
-          <t>finitial+last@lacasa.es (RocketReach 89.6%) (UNVERIFIED)</t>
+          <t>finitial+last@lacasa.es (RocketReach 89.6%) (UNVERIFIED) [VERIFIED: finitial+last is primary (RocketReach 89.6%)]</t>
         </is>
       </c>
     </row>
@@ -4289,7 +4289,7 @@
       </c>
       <c r="U44" s="2" t="inlineStr">
         <is>
-          <t>first.last@agoragp.com (RocketReach ~95%) (UNVERIFIED)</t>
+          <t>first.last@agoragp.com (RocketReach ~95%) (UNVERIFIED) [VERIFIED: first.last confirmed 95.3%; RRHH contact Sara Repolles]</t>
         </is>
       </c>
     </row>
@@ -4367,7 +4367,7 @@
       </c>
       <c r="T45" s="2" t="inlineStr">
         <is>
-          <t>info@forestalia.com; contabilidad@forestalia.com</t>
+          <t>info@forestalia.com; contabilidad@forestalia.com; rrhh@forestalia.com (HR mailbox, published on Unete page); lopd@forestalia.es</t>
         </is>
       </c>
       <c r="U45" s="2" t="inlineStr">
@@ -4621,7 +4621,7 @@
       </c>
       <c r="U48" s="2" t="inlineStr">
         <is>
-          <t>finitial.last@libelium.com (RocketReach 88.2%) (UNVERIFIED)</t>
+          <t>finitial.last@libelium.com (RocketReach 88.2%) (UNVERIFIED) [CORRECTED: pattern is first.lastinitial@libelium.com (e.g. jane.d@), not finitial.last]</t>
         </is>
       </c>
     </row>
@@ -4998,7 +4998,7 @@
       </c>
       <c r="T54" s="2" t="inlineStr">
         <is>
-          <t>victor.martinez@tsbzaragoza.com; administracion@tsbzaragoza.com (Laftur now trades as TSB Zaragoza)</t>
+          <t>victor.martinez@tsbzaragoza.com; administracion@tsbzaragoza.com (Laftur now trades as TSB Zaragoza); victor.martinez@tsbzaragoza.com; administracion@tsbzaragoza.com (med-confidence)</t>
         </is>
       </c>
       <c r="U54" s="2" t="inlineStr">
@@ -5293,7 +5293,7 @@
       </c>
       <c r="T59" s="2" t="inlineStr">
         <is>
-          <t>maetel@maetel.com; protecciondedatos@maetel.com</t>
+          <t>maetel@maetel.com; protecciondedatos@maetel.com; personal@maetel.com (CV/empleo box)</t>
         </is>
       </c>
       <c r="U59" s="2" t="inlineStr">
@@ -5405,7 +5405,7 @@
       </c>
       <c r="U60" s="2" t="inlineStr">
         <is>
-          <t>fernando.lecinena@lecitrailer.es / flecinena@lecitrailer.es — first.last or finitial+last per RocketReach masks (UNVERIFIED)</t>
+          <t>fernando.lecinena@lecitrailer.es / flecinena@lecitrailer.es — first.last or finitial+last per RocketReach masks (UNVERIFIED) [CORRECTED: pattern is firstlast -&gt; fernandolecinena@lecitrailer.es, not first.last/flecinena@]</t>
         </is>
       </c>
     </row>
@@ -5512,7 +5512,7 @@
       </c>
       <c r="U61" s="2" t="inlineStr">
         <is>
-          <t>first.last@hmy-group.com (ContactOut) (UNVERIFIED)</t>
+          <t>first.last@hmy-group.com (ContactOut) (UNVERIFIED) [VERIFIED: first.last@hmy-group.com ~99%; now part of ITAB]</t>
         </is>
       </c>
     </row>
@@ -5619,7 +5619,7 @@
       </c>
       <c r="U62" s="2" t="inlineStr">
         <is>
-          <t>first.last@samca.com (SAMCA group convention) (UNVERIFIED)</t>
+          <t>first.last@samca.com (SAMCA group convention) (UNVERIFIED) [VERIFIED: staff use @samca.com not @novapet.com]</t>
         </is>
       </c>
     </row>
@@ -5721,12 +5721,12 @@
       </c>
       <c r="T63" s="2" t="inlineStr">
         <is>
-          <t>info@megasa.com</t>
+          <t>info@megasa.com; batienza@megasa.es (eInforma)</t>
         </is>
       </c>
       <c r="U63" s="2" t="inlineStr">
         <is>
-          <t>eduardo.pinera@megasa.com — first.last (corporate megasa.com, n-&gt;n) (UNVERIFIED)</t>
+          <t>eduardo.pinera@megasa.com — first.last (corporate megasa.com, n-&gt;n) (UNVERIFIED) [CORRECTED: domain is megasa.es, finitial+last -&gt; epinera@megasa.es (batienza@megasa.es confirmed)]</t>
         </is>
       </c>
     </row>
@@ -5825,7 +5825,7 @@
       </c>
       <c r="U64" s="2" t="inlineStr">
         <is>
-          <t>first.last@grupocarreras.com (RocketReach 72.7%, e.g. alberto.borque@) (UNVERIFIED)</t>
+          <t>first.last@grupocarreras.com (RocketReach 72.7%, e.g. alberto.borque@) (UNVERIFIED) [VERIFIED: first.last confirmed (alberto.borque@)]</t>
         </is>
       </c>
     </row>
@@ -5919,7 +5919,7 @@
       </c>
       <c r="T65" s="2" t="inlineStr">
         <is>
-          <t>comunicacion.spain@adidas.com (corporate domain adidas.com)</t>
+          <t>comunicacion.spain@adidas.com (corporate domain adidas.com); comunicacion.spain@adidas.com</t>
         </is>
       </c>
       <c r="U65" s="2" t="inlineStr">
@@ -6328,7 +6328,7 @@
       </c>
       <c r="U69" s="2" t="inlineStr">
         <is>
-          <t>first.last@valeo.com (RocketReach 97.9%) (UNVERIFIED)</t>
+          <t>first.last@valeo.com (RocketReach 97.9%) (UNVERIFIED) [VERIFIED: first.last@valeo.com ~98%]</t>
         </is>
       </c>
     </row>
@@ -6418,12 +6418,12 @@
       </c>
       <c r="T70" s="2" t="inlineStr">
         <is>
-          <t>None found verbatim</t>
+          <t>None found verbatim; adolfo.bernad@eu.fujikura.com; francisco.espasa@eu.fujikura.com</t>
         </is>
       </c>
       <c r="U70" s="2" t="inlineStr">
         <is>
-          <t>finitial+last@fujikura-automotive.com (RocketReach 100%) (UNVERIFIED)</t>
+          <t>finitial+last@fujikura-automotive.com (RocketReach 100%) (UNVERIFIED) [CORRECTED: first.last@eu.fujikura.com (adolfo.bernad@, francisco.espasa@ confirmed)]</t>
         </is>
       </c>
     </row>
@@ -6513,12 +6513,12 @@
       </c>
       <c r="T71" s="2" t="inlineStr">
         <is>
-          <t>None found verbatim</t>
+          <t>None found verbatim; inma.ruiz@adient.com</t>
         </is>
       </c>
       <c r="U71" s="2" t="inlineStr">
         <is>
-          <t>first.last@adient.com (RocketReach 99.9%) (UNVERIFIED)</t>
+          <t>first.last@adient.com (RocketReach 99.9%) (UNVERIFIED) [VERIFIED: first.last@adient.com confirmed (inma.ruiz@)]</t>
         </is>
       </c>
     </row>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="T72" s="2" t="inlineStr">
         <is>
-          <t>None found verbatim</t>
+          <t>None found verbatim; comunicacion.es@schindler.com; schindler24.es@schindler.com</t>
         </is>
       </c>
       <c r="U72" s="2" t="inlineStr">
@@ -6703,7 +6703,7 @@
       </c>
       <c r="T73" s="2" t="inlineStr">
         <is>
-          <t>None found verbatim</t>
+          <t>None found verbatim; caf@caf.net; prensa@caf.net; dpo@caf.net</t>
         </is>
       </c>
       <c r="U73" s="2" t="inlineStr">
@@ -6901,7 +6901,7 @@
       </c>
       <c r="T75" s="2" t="inlineStr">
         <is>
-          <t>secretariageneral@ibercaja.es; atencioncliente@ibercaja.es</t>
+          <t>secretariageneral@ibercaja.es; atencioncliente@ibercaja.es; comunicacion@ibercaja.es</t>
         </is>
       </c>
       <c r="U75" s="2" t="inlineStr">
@@ -7000,7 +7000,7 @@
       </c>
       <c r="T76" s="2" t="inlineStr">
         <is>
-          <t>None found verbatim</t>
+          <t>None found verbatim; comunicacion@inditex.com</t>
         </is>
       </c>
       <c r="U76" s="2" t="inlineStr">
@@ -7198,7 +7198,7 @@
       </c>
       <c r="T78" s="2" t="inlineStr">
         <is>
-          <t>None found verbatim</t>
+          <t>None found verbatim; contactgdpr@tereos.com</t>
         </is>
       </c>
       <c r="U78" s="2" t="inlineStr">
@@ -7510,10 +7510,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr"/>
-    </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>

</xml_diff>